<commit_message>
Daily NSE scan: 2026-09-22
</commit_message>
<xml_diff>
--- a/output/2026-09-22/enriched_analysis.xlsx
+++ b/output/2026-09-22/enriched_analysis.xlsx
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>3.641</v>
+        <v>3.626</v>
       </c>
       <c r="W2" t="n">
-        <v>2909</v>
+        <v>2921</v>
       </c>
       <c r="X2" t="n">
-        <v>22.8</v>
+        <v>22.9</v>
       </c>
       <c r="Y2" t="n">
         <v>75</v>
@@ -1161,13 +1161,13 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>0.051</v>
+        <v>0.05</v>
       </c>
       <c r="W3" t="n">
-        <v>2629</v>
+        <v>2630</v>
       </c>
       <c r="X3" t="n">
-        <v>9.01</v>
+        <v>9.02</v>
       </c>
       <c r="Y3" t="n">
         <v>36</v>
@@ -1393,13 +1393,13 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>0.914</v>
+        <v>0.919</v>
       </c>
       <c r="W4" t="n">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="X4" t="n">
-        <v>8.98</v>
+        <v>8.93</v>
       </c>
       <c r="Y4" t="n">
         <v>17</v>
@@ -1625,13 +1625,13 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>0.289</v>
+        <v>0.293</v>
       </c>
       <c r="W5" t="n">
-        <v>1060</v>
+        <v>1045</v>
       </c>
       <c r="X5" t="n">
-        <v>10.4</v>
+        <v>10.2</v>
       </c>
       <c r="Y5" t="n">
         <v>7</v>
@@ -2047,25 +2047,25 @@
         <v>662.75</v>
       </c>
       <c r="J7" t="n">
-        <v>625.41</v>
+        <v>630.67</v>
       </c>
       <c r="K7" t="n">
-        <v>6</v>
+        <v>5.1</v>
       </c>
       <c r="L7" t="n">
         <v>64.68000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>3.96</v>
+        <v>4.7</v>
       </c>
       <c r="N7" t="n">
-        <v>39558097</v>
+        <v>46955184</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>39558097</v>
+        <v>46955184</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
@@ -2079,15 +2079,15 @@
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>21-09-2026</t>
         </is>
       </c>
       <c r="V7" t="n">
-        <v>0.323</v>
+        <v>0.384</v>
       </c>
       <c r="W7" t="n">
         <v>1224</v>
@@ -2129,10 +2129,10 @@
         <v>43</v>
       </c>
       <c r="AJ7" t="n">
-        <v>625.4145705206241</v>
+        <v>630.668797765033</v>
       </c>
       <c r="AK7" t="n">
-        <v>6</v>
+        <v>5.1</v>
       </c>
       <c r="AL7" t="inlineStr">
         <is>
@@ -2156,47 +2156,47 @@
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>21-09-2026</t>
         </is>
       </c>
       <c r="AQ7" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="AR7" t="n">
         <v>95</v>
       </c>
       <c r="AS7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT7" t="n">
         <v>4</v>
       </c>
-      <c r="AT7" t="n">
-        <v>3</v>
-      </c>
       <c r="AU7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AV7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="AW7" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="AX7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="AY7" t="n">
-        <v>6266479</v>
+        <v>13663566</v>
       </c>
       <c r="AZ7" t="n">
-        <v>9395107</v>
+        <v>16792194</v>
       </c>
       <c r="BA7" t="n">
-        <v>22368301</v>
+        <v>29765388</v>
       </c>
       <c r="BB7" t="n">
-        <v>28676708</v>
+        <v>36073795</v>
       </c>
       <c r="BC7" t="n">
-        <v>31585748</v>
+        <v>38982835</v>
       </c>
       <c r="BD7" t="n">
         <v>0</v>
@@ -2229,10 +2229,10 @@
         <v>0</v>
       </c>
       <c r="BN7" t="n">
-        <v>6266479</v>
+        <v>13663566</v>
       </c>
       <c r="BO7" t="n">
-        <v>22368301</v>
+        <v>29765388</v>
       </c>
       <c r="BP7" t="n">
         <v>2</v>
@@ -2241,7 +2241,7 @@
         <v>0</v>
       </c>
       <c r="BR7" t="n">
-        <v>0.2801</v>
+        <v>0.459</v>
       </c>
     </row>
     <row r="8">
@@ -2319,13 +2319,13 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0.053</v>
+        <v>0.054</v>
       </c>
       <c r="W8" t="n">
-        <v>1538</v>
+        <v>1521</v>
       </c>
       <c r="X8" t="n">
-        <v>20.7</v>
+        <v>20.5</v>
       </c>
       <c r="Y8" t="n">
         <v>55</v>
@@ -2551,13 +2551,13 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.534</v>
       </c>
       <c r="W9" t="n">
-        <v>324</v>
+        <v>338</v>
       </c>
       <c r="X9" t="n">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="Y9" t="n">
         <v>22</v>
@@ -2786,10 +2786,10 @@
         <v>0.111</v>
       </c>
       <c r="W10" t="n">
-        <v>2840</v>
+        <v>2819</v>
       </c>
       <c r="X10" t="n">
-        <v>24.9</v>
+        <v>24.7</v>
       </c>
       <c r="Y10" t="n">
         <v>-3</v>
@@ -3018,7 +3018,7 @@
         <v>0.367</v>
       </c>
       <c r="W11" t="n">
-        <v>2645</v>
+        <v>2646</v>
       </c>
       <c r="X11" t="n">
         <v>21.7</v>
@@ -3247,13 +3247,13 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>2.28</v>
+        <v>2.267</v>
       </c>
       <c r="W12" t="n">
-        <v>2613</v>
+        <v>2628</v>
       </c>
       <c r="X12" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="Y12" t="n">
         <v>6</v>
@@ -3479,13 +3479,13 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>0.155</v>
+        <v>0.16</v>
       </c>
       <c r="W13" t="n">
-        <v>715</v>
+        <v>694</v>
       </c>
       <c r="X13" t="n">
-        <v>59.8</v>
+        <v>58</v>
       </c>
       <c r="Y13" t="n">
         <v>3</v>
@@ -3714,10 +3714,10 @@
         <v>0.046</v>
       </c>
       <c r="W14" t="n">
-        <v>15704</v>
+        <v>15755</v>
       </c>
       <c r="X14" t="n">
-        <v>40</v>
+        <v>40.1</v>
       </c>
       <c r="Y14" t="n">
         <v>83</v>
@@ -3943,10 +3943,10 @@
         </is>
       </c>
       <c r="V15" t="n">
-        <v>1.582</v>
+        <v>1.595</v>
       </c>
       <c r="W15" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="X15" t="inlineStr"/>
       <c r="Y15" t="n">
@@ -4173,10 +4173,10 @@
         </is>
       </c>
       <c r="V16" t="n">
-        <v>0.102</v>
+        <v>0.101</v>
       </c>
       <c r="W16" t="n">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="X16" t="n">
         <v>27</v>
@@ -4405,13 +4405,13 @@
         </is>
       </c>
       <c r="V17" t="n">
-        <v>0.489</v>
+        <v>0.496</v>
       </c>
       <c r="W17" t="n">
-        <v>694</v>
+        <v>685</v>
       </c>
       <c r="X17" t="n">
-        <v>15.3</v>
+        <v>15</v>
       </c>
       <c r="Y17" t="n">
         <v>-1</v>
@@ -4872,10 +4872,10 @@
         <v>0.06900000000000001</v>
       </c>
       <c r="W19" t="n">
-        <v>819</v>
+        <v>822</v>
       </c>
       <c r="X19" t="n">
-        <v>20.7</v>
+        <v>20.8</v>
       </c>
       <c r="Y19" t="n">
         <v>19</v>
@@ -5099,13 +5099,13 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>0.44</v>
+        <v>0.436</v>
       </c>
       <c r="W20" t="n">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="X20" t="n">
-        <v>39</v>
+        <v>39.4</v>
       </c>
       <c r="Y20" t="n">
         <v>21</v>
@@ -5331,13 +5331,13 @@
         </is>
       </c>
       <c r="V21" t="n">
-        <v>0.291</v>
+        <v>0.294</v>
       </c>
       <c r="W21" t="n">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="X21" t="n">
-        <v>25.4</v>
+        <v>25.1</v>
       </c>
       <c r="Y21" t="n">
         <v>12</v>
@@ -5563,13 +5563,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>0.134</v>
+        <v>0.136</v>
       </c>
       <c r="W22" t="n">
-        <v>371</v>
+        <v>365</v>
       </c>
       <c r="X22" t="n">
-        <v>5.98</v>
+        <v>5.88</v>
       </c>
       <c r="Y22" t="n">
         <v>118</v>
@@ -5791,13 +5791,13 @@
         </is>
       </c>
       <c r="V23" t="n">
-        <v>1.752</v>
+        <v>1.741</v>
       </c>
       <c r="W23" t="n">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="X23" t="n">
-        <v>25.2</v>
+        <v>25.3</v>
       </c>
       <c r="Y23" t="n">
         <v>30</v>
@@ -6020,10 +6020,10 @@
         <v>0.007</v>
       </c>
       <c r="W24" t="n">
-        <v>5581</v>
+        <v>5587</v>
       </c>
       <c r="X24" t="n">
-        <v>9.449999999999999</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="Y24" t="n">
         <v>43</v>
@@ -6484,10 +6484,10 @@
         <v>0.054</v>
       </c>
       <c r="W26" t="n">
-        <v>2053</v>
+        <v>2033</v>
       </c>
       <c r="X26" t="n">
-        <v>47.1</v>
+        <v>46.7</v>
       </c>
       <c r="Y26" t="n">
         <v>20</v>
@@ -6945,13 +6945,13 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.636</v>
+        <v>0.646</v>
       </c>
       <c r="W28" t="n">
-        <v>369</v>
+        <v>363</v>
       </c>
       <c r="X28" t="n">
-        <v>1190</v>
+        <v>1170</v>
       </c>
       <c r="Y28" t="n">
         <v>-61</v>
@@ -7176,7 +7176,7 @@
         <v>0.095</v>
       </c>
       <c r="W29" t="n">
-        <v>1555</v>
+        <v>1554</v>
       </c>
       <c r="X29" t="n">
         <v>14.1</v>
@@ -7408,7 +7408,7 @@
         <v>0.026</v>
       </c>
       <c r="W30" t="n">
-        <v>941</v>
+        <v>944</v>
       </c>
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="n">
@@ -7635,13 +7635,13 @@
         </is>
       </c>
       <c r="V31" t="n">
-        <v>0.963</v>
+        <v>0.931</v>
       </c>
       <c r="W31" t="n">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="X31" t="n">
-        <v>6.03</v>
+        <v>6.24</v>
       </c>
       <c r="Y31" t="n">
         <v>31</v>
@@ -7863,13 +7863,13 @@
         </is>
       </c>
       <c r="V32" t="n">
-        <v>0.053</v>
+        <v>0.052</v>
       </c>
       <c r="W32" t="n">
-        <v>5001</v>
+        <v>5010</v>
       </c>
       <c r="X32" t="n">
-        <v>32.6</v>
+        <v>32.7</v>
       </c>
       <c r="Y32" t="n">
         <v>-25</v>
@@ -8098,10 +8098,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W33" t="n">
-        <v>52703</v>
+        <v>52528</v>
       </c>
       <c r="X33" t="n">
-        <v>44.6</v>
+        <v>44.5</v>
       </c>
       <c r="Y33" t="n">
         <v>5</v>
@@ -8559,13 +8559,13 @@
         </is>
       </c>
       <c r="V35" t="n">
-        <v>0.479</v>
+        <v>0.486</v>
       </c>
       <c r="W35" t="n">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="X35" t="n">
-        <v>11.4</v>
+        <v>11.3</v>
       </c>
       <c r="Y35" t="n">
         <v>19</v>
@@ -8791,13 +8791,13 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="W36" t="n">
-        <v>767</v>
+        <v>756</v>
       </c>
       <c r="X36" t="n">
-        <v>13.9</v>
+        <v>13.7</v>
       </c>
       <c r="Y36" t="n">
         <v>185</v>
@@ -9024,10 +9024,10 @@
         <v>0</v>
       </c>
       <c r="W37" t="n">
-        <v>3939</v>
+        <v>3926</v>
       </c>
       <c r="X37" t="n">
-        <v>88.7</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="Y37" t="n">
         <v>42</v>
@@ -9256,7 +9256,7 @@
         <v>0.021</v>
       </c>
       <c r="W38" t="n">
-        <v>9372</v>
+        <v>9414</v>
       </c>
       <c r="X38" t="n">
         <v>12.4</v>
@@ -9488,10 +9488,10 @@
         <v>0.033</v>
       </c>
       <c r="W39" t="n">
-        <v>730</v>
+        <v>744</v>
       </c>
       <c r="X39" t="n">
-        <v>47.6</v>
+        <v>48.5</v>
       </c>
       <c r="Y39" t="n">
         <v>7</v>
@@ -9717,13 +9717,13 @@
         </is>
       </c>
       <c r="V40" t="n">
-        <v>0.546</v>
+        <v>0.547</v>
       </c>
       <c r="W40" t="n">
-        <v>3540</v>
+        <v>3535</v>
       </c>
       <c r="X40" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="Y40" t="n">
         <v>2</v>
@@ -9952,10 +9952,10 @@
         <v>0</v>
       </c>
       <c r="W41" t="n">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="X41" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="Y41" t="n">
         <v>5</v>
@@ -10184,7 +10184,7 @@
         <v>0.128</v>
       </c>
       <c r="W42" t="n">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="X42" t="n">
         <v>13.8</v>
@@ -10411,13 +10411,13 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.203</v>
+        <v>0.207</v>
       </c>
       <c r="W43" t="n">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="X43" t="n">
-        <v>26.3</v>
+        <v>25.8</v>
       </c>
       <c r="Y43" t="n">
         <v>21</v>
@@ -10646,7 +10646,7 @@
         <v>0.223</v>
       </c>
       <c r="W44" t="n">
-        <v>1787</v>
+        <v>1789</v>
       </c>
       <c r="X44" t="n">
         <v>18.9</v>
@@ -10875,13 +10875,13 @@
         </is>
       </c>
       <c r="V45" t="n">
-        <v>0.042</v>
+        <v>0.041</v>
       </c>
       <c r="W45" t="n">
-        <v>1669</v>
+        <v>1680</v>
       </c>
       <c r="X45" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="Y45" t="n">
         <v>10</v>
@@ -11107,13 +11107,13 @@
         </is>
       </c>
       <c r="V46" t="n">
-        <v>0.128</v>
+        <v>0.129</v>
       </c>
       <c r="W46" t="n">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="X46" t="n">
-        <v>26.6</v>
+        <v>26.3</v>
       </c>
       <c r="Y46" t="n">
         <v>9</v>
@@ -11339,13 +11339,13 @@
         </is>
       </c>
       <c r="V47" t="n">
-        <v>0.256</v>
+        <v>0.259</v>
       </c>
       <c r="W47" t="n">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="X47" t="n">
-        <v>14.5</v>
+        <v>14.3</v>
       </c>
       <c r="Y47" t="n">
         <v>16</v>
@@ -11574,10 +11574,10 @@
         <v>0</v>
       </c>
       <c r="W48" t="n">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="X48" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="Y48" t="n">
         <v>3</v>
@@ -11806,7 +11806,7 @@
         <v>0</v>
       </c>
       <c r="W49" t="n">
-        <v>8961</v>
+        <v>8942</v>
       </c>
       <c r="X49" t="n">
         <v>15.2</v>
@@ -12035,13 +12035,13 @@
         </is>
       </c>
       <c r="V50" t="n">
-        <v>0.355</v>
+        <v>0.356</v>
       </c>
       <c r="W50" t="n">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="X50" t="n">
-        <v>97.5</v>
+        <v>97.3</v>
       </c>
       <c r="Y50" t="n">
         <v>246</v>
@@ -12270,7 +12270,7 @@
         <v>0.081</v>
       </c>
       <c r="W51" t="n">
-        <v>1686</v>
+        <v>1684</v>
       </c>
       <c r="X51" t="n">
         <v>30.4</v>
@@ -12502,10 +12502,10 @@
         <v>0</v>
       </c>
       <c r="W52" t="n">
-        <v>116392</v>
+        <v>116622</v>
       </c>
       <c r="X52" t="n">
-        <v>33.5</v>
+        <v>33.6</v>
       </c>
       <c r="Y52" t="n">
         <v>18</v>
@@ -12918,23 +12918,23 @@
         <v>662.75</v>
       </c>
       <c r="D7" t="n">
-        <v>625.41</v>
+        <v>630.67</v>
       </c>
       <c r="E7" t="n">
-        <v>6</v>
+        <v>5.1</v>
       </c>
       <c r="F7" t="n">
         <v>64.68000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>3.96</v>
+        <v>4.7</v>
       </c>
       <c r="H7" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>21-09-2026</t>
         </is>
       </c>
     </row>

</xml_diff>